<commit_message>
Fill verified emails for the 10 added mortgage contacts
All 10 resolved and verified for 9 Apollo credits.

Worth noting for future runs: guessing a surname from Apollo's mask and
passing it to --targets is unreliable - 7 of 10 guesses were wrong
(Houston not Horan, Kaspar not Kaiser, Luechauer not Luster, Schaub not
Schwab, Hansen not Hanson, Redding not Reding, Baker not Barker). Matching
on the mask itself and letting the enrichment return the real name is the
correct approach, and is what recovered all six misses.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WA3eMoHLG5tHsDy3VcGJJG
</commit_message>
<xml_diff>
--- a/mortgage_reviewed.xlsx
+++ b/mortgage_reviewed.xlsx
@@ -59,14 +59,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00DDEBF7"/>
+        <bgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
-        <bgColor rgb="00DDEBF7"/>
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -95,8 +95,8 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -466,12 +466,12 @@
   <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -546,147 +546,155 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
+          <t>Jennifer Houston</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>SVP</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>jhouston@cmgfi.com</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>senior exec in corridor</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>CMG Home Loans</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
           <t>Phil George</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Marketing Director</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>pgeorge@cmgfi.com</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>KEEP</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>top marketing at this company</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>top marketing</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>CMG Home Loans</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>John Weaver</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Marketing Manager</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>jweaver@cmgfi.com</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>KEEP</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>marketing</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>CMG Home Loans</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Michele Sniffen</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Processing Manager</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>msniffen@cmgfi.com</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>RED</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>RED</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>back office - not exec/VP/director or marketing</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>CMG Home Loans</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Jennifer Ho***n</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>SVP</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr"/>
-      <c r="E6" s="4" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>DHI Mortgage Co. Ltd.</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Sonya Luechauer</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>President and Chief Executive Officer</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>sluechauer@dhimortgage.com</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>ADD</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>senior exec in corridor</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>DHI Mortgage Co. Ltd.</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Monica Ka***r</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>AVP, National Marketing Manager</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr"/>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>highest marketing at DHI</t>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>C-level, in corridor</t>
         </is>
       </c>
     </row>
@@ -698,59 +706,59 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
+          <t>Monica Kaspar</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>AVP, National Marketing Manager</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>makaspar@dhimortgage.com</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>highest marketing at DHI</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>DHI Mortgage Co. Ltd.</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
           <t>Thomas VanBuskirk</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Digital Marketing Manager</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>tvanbuskirk@dhimortgage.com</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>KEEP</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>marketing - NOTE your sheet lists him as branch sales manager, Apollo says Digital Marketing Manager</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>DHI Mortgage Co. Ltd.</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Viky Kalyta</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Marketing Coordinator</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>vkalyta@dhimortgage.com</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>KEEP</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>marketing, lowest rank of the three</t>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>marketing - your sheet says branch sales manager, Apollo says Digital Marketing Manager</t>
         </is>
       </c>
     </row>
@@ -762,23 +770,27 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Sonya Lu***r</t>
+          <t>Viky Kalyta</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>President and Chief Executive Officer</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr"/>
+          <t>Marketing Coordinator</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>vkalyta@dhimortgage.com</t>
+        </is>
+      </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>ADD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>C-level, in corridor</t>
+          <t>marketing, lowest of the three</t>
         </is>
       </c>
     </row>
@@ -822,27 +834,27 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Andrew Brock</t>
+          <t>Greg Schaub</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>South region head, private bank</t>
+          <t>EVP Sales</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>andrew.j.brock@jpmorgan.com</t>
+          <t>greg.schaub@chase.com</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>KEEP</t>
+          <t>ADD</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>regional head</t>
+          <t>EVP in corridor</t>
         </is>
       </c>
     </row>
@@ -854,23 +866,27 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Greg Sc***b</t>
+          <t>Andrew Brock</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>EVP Sales</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr"/>
+          <t>South region head, private bank</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>andrew.j.brock@jpmorgan.com</t>
+        </is>
+      </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>ADD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>EVP in corridor</t>
+          <t>regional head</t>
         </is>
       </c>
     </row>
@@ -971,32 +987,32 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Lennar Mortgage</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Kyle Simpson</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>SVP, Regional Manager</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>KyleSimpson@lennarmortgage.com</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>KEEP</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>SVP - your sheet had no title, Apollo confirms</t>
         </is>
@@ -1067,58 +1083,66 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Fairway Independent Mortgage</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Chandler Ha***n</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Matt Wood</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Managing Partner</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>mwood@fairwaymc.com</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>exec in corridor</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Fairway Independent Mortgage</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Chandler Hansen</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>Marketing Manager</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr"/>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>chandler.hansen@fairwaymc.com</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>ADD</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>top marketing in corridor</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Fairway Independent Mortgage</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Matt Wo***d</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Managing Partner</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr"/>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>exec in corridor</t>
         </is>
       </c>
     </row>
@@ -1182,7 +1206,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>loan officer - not exec/VP/director or marketing</t>
+          <t>loan officer</t>
         </is>
       </c>
     </row>
@@ -1283,122 +1307,130 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>LoanPeople</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>Max Leaman</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>max.leaman@loanpeople.com</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>KEEP</t>
         </is>
       </c>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>C-level</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>LoanPeople</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Dana Leaman</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>CMO</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>Dana@maxleaman.com</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
         <is>
           <t>KEEP</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="F28" s="4" t="inlineStr">
         <is>
           <t>top marketing - CMO</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>Pulte Mortgage LLC</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Stephanie Re***g</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Pablo Rivas</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Division President</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>pablo.rivas@pultegroup.com</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>ADD</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>president</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Pulte Mortgage LLC</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Stephanie Redding</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>Director of Marketing</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr"/>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>stephanie.redding@pultegroup.com</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
         <is>
           <t>ADD</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="F30" s="3" t="inlineStr">
         <is>
           <t>top marketing in corridor</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>Pulte Mortgage LLC</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>Pablo Rivas</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Division president</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr"/>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>ADD</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>president - needs email, Apollo has him</t>
         </is>
       </c>
     </row>
@@ -1431,30 +1463,34 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>KBHS Home Loans LLC</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>Louie Colatriano</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>President</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr"/>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>lcolatriano1@kbhshomeloans.com</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
         <is>
           <t>ADD</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>president - needs email</t>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>president</t>
         </is>
       </c>
     </row>
@@ -1519,28 +1555,32 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>M/I Financial LLC</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>Derek Ba***r</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Derek Baker</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>Area President</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr"/>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>dbaker@mihomes.com</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
         <is>
           <t>ADD</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>president in corridor</t>
         </is>
@@ -1755,64 +1795,64 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="A43" s="4" t="inlineStr">
         <is>
           <t>Guild Mortgage Company LLC</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>Chad Overhauser</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr">
+      <c r="C43" s="4" t="inlineStr">
         <is>
           <t>Divisional VP (Apollo: SVP)</t>
         </is>
       </c>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="D43" s="4" t="inlineStr">
         <is>
           <t>coverhauser@guildmortgage.net</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="E43" s="4" t="inlineStr">
         <is>
           <t>KEEP</t>
         </is>
       </c>
-      <c r="F43" s="3" t="inlineStr">
+      <c r="F43" s="4" t="inlineStr">
         <is>
           <t>VP</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="inlineStr">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>Guild Mortgage Company LLC</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr">
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>Eric Weiss</t>
         </is>
       </c>
-      <c r="C44" s="3" t="inlineStr">
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>RVP (Apollo: SVP)</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr">
+      <c r="D44" s="4" t="inlineStr">
         <is>
           <t>eweiss@guildmortgage.net</t>
         </is>
       </c>
-      <c r="E44" s="3" t="inlineStr">
+      <c r="E44" s="4" t="inlineStr">
         <is>
           <t>KEEP</t>
         </is>
       </c>
-      <c r="F44" s="3" t="inlineStr">
+      <c r="F44" s="4" t="inlineStr">
         <is>
           <t>VP</t>
         </is>
@@ -1834,7 +1874,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="64" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1857,7 +1897,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>only IT/security/ops VPs in corridor - no relevant POC</t>
+          <t>only IT/security/ops VPs in corridor - right seniority, wrong function</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1921,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>only engineering VPs in corridor - no relevant POC</t>
+          <t>only engineering VPs in corridor</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1981,7 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>only an Associate Director of Strategic Ops - weak</t>
+          <t>only an Associate Director of Strategic Ops</t>
         </is>
       </c>
     </row>
@@ -1965,7 +2005,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>nobody in corridor at this domain</t>
+          <t>nobody in the corridor at this domain</t>
         </is>
       </c>
     </row>
@@ -1984,7 +2024,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="64" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2007,7 +2047,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Confirmed - fits your rules, keep as-is</t>
+          <t>Confirmed - already in your data and fits the rules</t>
         </is>
       </c>
     </row>
@@ -2019,7 +2059,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Added by me - correct title found in Apollo, email still needed</t>
+          <t>Added by me - all verified emails</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2071,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Not the best POC - see Reason column</t>
+          <t>Not the best POC - see Reason</t>
         </is>
       </c>
     </row>

</xml_diff>